<commit_message>
#51 Completed and Delievrable generated
</commit_message>
<xml_diff>
--- a/Design Files/Powermodule-v10.1.0/Deliverables/BOM/Client_BOM_Powermodule-v9.0.0.xlsx
+++ b/Design Files/Powermodule-v10.1.0/Deliverables/BOM/Client_BOM_Powermodule-v9.0.0.xlsx
@@ -1,20 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Powermodule-v10.0.0\Deliverables\BOM\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19635" windowHeight="7620"/>
+    <workbookView windowWidth="19635" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -55,9 +50,15 @@
     <t>Manufacturer</t>
   </si>
   <si>
+    <t>Value</t>
+  </si>
+  <si>
     <t>Quantity</t>
   </si>
   <si>
+    <t>Remarks</t>
+  </si>
+  <si>
     <t>Capacitor</t>
   </si>
   <si>
@@ -484,6 +485,9 @@
     <t>DNP</t>
   </si>
   <si>
+    <t>Do Not Place</t>
+  </si>
+  <si>
     <t>TEST POINT</t>
   </si>
   <si>
@@ -1082,22 +1086,19 @@
   </si>
   <si>
     <t>CR927</t>
-  </si>
-  <si>
-    <t>Remarks</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Do Not Place</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="15">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="34">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1149,6 +1150,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <strike/>
       <sz val="10"/>
       <color rgb="FFFF0000"/>
@@ -1182,6 +1190,7 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <strike/>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -1193,26 +1202,162 @@
       <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <strike/>
-      <sz val="9"/>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <family val="2"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1231,8 +1376,194 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="8">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -1323,9 +1654,251 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="7" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
   <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1365,61 +1938,105 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Hyperlink" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
-      <color rgb="FF03A4CB"/>
-      <color rgb="FF2CD0B2"/>
+      <color rgb="0003A4CB"/>
+      <color rgb="002CD0B2"/>
     </mruColors>
   </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1677,32 +2294,31 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R78"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="3.14285714285714" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.7142857142857" style="2" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="29.42578125" customWidth="1"/>
-    <col min="13" max="13" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.5714285714286" customWidth="1"/>
+    <col min="7" max="7" width="33.4285714285714" customWidth="1"/>
+    <col min="8" max="8" width="21.4285714285714" customWidth="1"/>
+    <col min="9" max="9" width="9.42857142857143" customWidth="1"/>
+    <col min="10" max="10" width="8.71428571428571" customWidth="1"/>
+    <col min="11" max="11" width="29.4285714285714" customWidth="1"/>
+    <col min="13" max="13" width="10.5714285714286" customWidth="1"/>
+    <col min="14" max="14" width="25.2857142857143" customWidth="1"/>
+    <col min="15" max="15" width="8.71428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" thickBot="1">
+    <row r="1" ht="15.75" spans="1:11">
       <c r="A1" s="3"/>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1711,11 +2327,11 @@
       <c r="F1" s="5"/>
       <c r="G1" s="5"/>
       <c r="H1" s="5"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-    </row>
-    <row r="2" spans="1:11" ht="15.75" thickBot="1">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+      <c r="K1" s="25"/>
+    </row>
+    <row r="2" ht="15.75" spans="1:11">
       <c r="A2" s="3"/>
       <c r="B2" s="6" t="s">
         <v>0</v>
@@ -1739,816 +2355,816 @@
         <v>6</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>351</v>
+        <v>7</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="36.75" thickBot="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="36.75" spans="1:11">
       <c r="A3" s="3"/>
       <c r="B3" s="8">
         <f t="shared" ref="B3:B34" si="0">ROW(B3)-ROW($B$2)</f>
         <v>1</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J3" s="10">
         <v>4</v>
       </c>
       <c r="K3" s="10"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" thickBot="1">
+    <row r="4" ht="15.75" spans="1:11">
       <c r="A4" s="3"/>
       <c r="B4" s="8">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I4" s="13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J4" s="12">
         <v>8</v>
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" spans="1:11" ht="24.75" thickBot="1">
+    <row r="5" ht="24.75" spans="1:11">
       <c r="A5" s="3"/>
       <c r="B5" s="8">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="J5" s="10">
         <v>20</v>
       </c>
       <c r="K5" s="10"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" thickBot="1">
+    <row r="6" ht="15.75" spans="1:11">
       <c r="A6" s="3"/>
       <c r="B6" s="8">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G6" s="13" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H6" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J6" s="12">
         <v>2</v>
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" spans="1:11" ht="15.75" thickBot="1">
+    <row r="7" ht="15.75" spans="1:11">
       <c r="A7" s="3"/>
       <c r="B7" s="8">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J7" s="10">
         <v>6</v>
       </c>
       <c r="K7" s="10"/>
     </row>
-    <row r="8" spans="1:11" ht="36.75" thickBot="1">
+    <row r="8" ht="36.75" spans="1:11">
       <c r="A8" s="3"/>
       <c r="B8" s="8">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F8" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I8" s="13" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J8" s="12">
         <v>4</v>
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" spans="1:11" ht="15.75" thickBot="1">
+    <row r="9" ht="15.75" spans="1:11">
       <c r="A9" s="3"/>
       <c r="B9" s="8">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="10">
         <v>2</v>
       </c>
       <c r="K9" s="10"/>
     </row>
-    <row r="10" spans="1:11" ht="15.75" thickBot="1">
+    <row r="10" ht="15.75" spans="1:11">
       <c r="A10" s="3"/>
       <c r="B10" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F10" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G10" s="13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H10" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I10" s="13" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="J10" s="12">
         <v>4</v>
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" spans="1:11" ht="15.75" thickBot="1">
+    <row r="11" ht="15.75" spans="1:11">
       <c r="A11" s="3"/>
       <c r="B11" s="8">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="I11" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J11" s="10">
         <v>1</v>
       </c>
       <c r="K11" s="10"/>
     </row>
-    <row r="12" spans="1:11" ht="36.75" thickBot="1">
+    <row r="12" ht="36.75" spans="1:11">
       <c r="A12" s="3"/>
       <c r="B12" s="8">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E12" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I12" s="13" t="s">
         <v>57</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="G12" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="I12" s="13" t="s">
-        <v>55</v>
       </c>
       <c r="J12" s="12">
         <v>1</v>
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" spans="1:11" ht="15.75" thickBot="1">
+    <row r="13" ht="15.75" spans="1:11">
       <c r="A13" s="3"/>
       <c r="B13" s="8">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="I13" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J13" s="10">
         <v>2</v>
       </c>
       <c r="K13" s="10"/>
     </row>
-    <row r="14" spans="1:11" ht="24.75" thickBot="1">
+    <row r="14" ht="24.75" spans="1:11">
       <c r="A14" s="3"/>
       <c r="B14" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F14" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H14" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I14" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J14" s="12">
         <v>11</v>
       </c>
       <c r="K14" s="12"/>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1">
+    <row r="15" ht="15.75" spans="1:11">
       <c r="A15" s="3"/>
       <c r="B15" s="8">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="J15" s="10">
         <v>1</v>
       </c>
       <c r="K15" s="10"/>
     </row>
-    <row r="16" spans="1:11" ht="36.75" thickBot="1">
+    <row r="16" ht="24.75" spans="1:11">
       <c r="A16" s="3"/>
       <c r="B16" s="8">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D16" s="12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F16" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H16" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="I16" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J16" s="12">
         <v>8</v>
       </c>
       <c r="K16" s="12"/>
     </row>
-    <row r="17" spans="1:18" ht="24.75" thickBot="1">
+    <row r="17" ht="24.75" spans="1:11">
       <c r="A17" s="3"/>
       <c r="B17" s="8">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="E17" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>85</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="I17" s="11" t="s">
         <v>81</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>83</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>79</v>
       </c>
       <c r="J17" s="10">
         <v>2</v>
       </c>
       <c r="K17" s="10"/>
     </row>
-    <row r="18" spans="1:18" ht="24.75" thickBot="1">
+    <row r="18" ht="24.75" spans="1:11">
       <c r="A18" s="3"/>
       <c r="B18" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="I18" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J18" s="12">
         <v>1</v>
       </c>
       <c r="K18" s="12"/>
     </row>
-    <row r="19" spans="1:18" ht="15.75" thickBot="1">
+    <row r="19" ht="15.75" spans="1:11">
       <c r="A19" s="3"/>
       <c r="B19" s="8">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J19" s="10">
         <v>1</v>
       </c>
       <c r="K19" s="10"/>
     </row>
-    <row r="20" spans="1:18" ht="15.75" thickBot="1">
+    <row r="20" ht="15.75" spans="1:11">
       <c r="A20" s="3"/>
       <c r="B20" s="8">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F20" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I20" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J20" s="12">
         <v>2</v>
       </c>
       <c r="K20" s="12"/>
     </row>
-    <row r="21" spans="1:18" ht="15.75" thickBot="1">
+    <row r="21" ht="15.75" spans="1:11">
       <c r="A21" s="3"/>
       <c r="B21" s="8">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F21" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H21" s="10" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="I21" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J21" s="10">
         <v>1</v>
       </c>
       <c r="K21" s="10"/>
     </row>
-    <row r="22" spans="1:18" ht="15.75" thickBot="1">
+    <row r="22" ht="15.75" spans="1:11">
       <c r="A22" s="3"/>
       <c r="B22" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E22" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="H22" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="F22" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>107</v>
-      </c>
       <c r="I22" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J22" s="12">
         <v>1</v>
       </c>
       <c r="K22" s="12"/>
     </row>
-    <row r="23" spans="1:18" ht="24.75" thickBot="1">
+    <row r="23" ht="24.75" spans="1:11">
       <c r="A23" s="3"/>
       <c r="B23" s="8">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="E23" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H23" s="10" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I23" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J23" s="10">
         <v>4</v>
       </c>
       <c r="K23" s="10"/>
     </row>
-    <row r="24" spans="1:18" ht="15.75" thickBot="1">
+    <row r="24" ht="15.75" spans="1:11">
       <c r="A24" s="3"/>
       <c r="B24" s="8">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E24" s="13" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J24" s="12">
         <v>1</v>
       </c>
       <c r="K24" s="12"/>
     </row>
-    <row r="25" spans="1:18" ht="36.75" thickBot="1">
+    <row r="25" ht="36.75" spans="1:11">
       <c r="A25" s="3"/>
       <c r="B25" s="8">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F25" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="I25" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J25" s="10">
         <v>1</v>
       </c>
       <c r="K25" s="10"/>
     </row>
-    <row r="26" spans="1:18" ht="15.75" thickBot="1">
+    <row r="26" ht="15.75" spans="1:11">
       <c r="A26" s="3"/>
       <c r="B26" s="8">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F26" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G26" s="13" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H26" s="12" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I26" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J26" s="12">
         <v>1</v>
       </c>
       <c r="K26" s="12"/>
     </row>
-    <row r="27" spans="1:18" ht="36.75" thickBot="1">
+    <row r="27" ht="24.75" spans="1:11">
       <c r="A27" s="3"/>
       <c r="B27" s="8">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E27" s="11" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F27" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I27" s="11" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J27" s="10">
         <v>1</v>
       </c>
       <c r="K27" s="10"/>
     </row>
-    <row r="28" spans="1:18" ht="15.75" thickBot="1">
+    <row r="28" ht="15.75" spans="1:11">
       <c r="A28" s="3"/>
       <c r="B28" s="8">
         <f t="shared" si="0"/>
@@ -2556,126 +3172,126 @@
       </c>
       <c r="C28" s="14"/>
       <c r="D28" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E28" s="13" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F28" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G28" s="13" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="I28" s="13" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="J28" s="12">
         <v>1</v>
       </c>
       <c r="K28" s="12"/>
     </row>
-    <row r="29" spans="1:18" ht="24.75" thickBot="1">
+    <row r="29" ht="24.75" spans="1:11">
       <c r="A29" s="3"/>
       <c r="B29" s="8">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E29" s="11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J29" s="10">
         <v>3</v>
       </c>
       <c r="K29" s="10"/>
     </row>
-    <row r="30" spans="1:18" ht="24.75" thickBot="1">
+    <row r="30" ht="24.75" spans="1:11">
       <c r="A30" s="3"/>
       <c r="B30" s="8">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>140</v>
-      </c>
-      <c r="D30" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="E30" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="E30" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="H30" s="15" t="s">
         <v>147</v>
       </c>
-      <c r="F30" s="23" t="s">
-        <v>143</v>
-      </c>
-      <c r="G30" s="24" t="s">
-        <v>148</v>
-      </c>
-      <c r="H30" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="I30" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="J30" s="23">
+      <c r="I30" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J30" s="15">
         <v>1</v>
       </c>
-      <c r="K30" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="31" spans="1:18" s="1" customFormat="1" ht="48.75" thickBot="1">
-      <c r="A31" s="15"/>
-      <c r="B31" s="16">
+      <c r="K30" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" s="1" customFormat="1" ht="48.75" spans="1:18">
+      <c r="A31" s="17"/>
+      <c r="B31" s="18">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C31" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="D31" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="E31" s="19" t="s">
+      <c r="C31" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>154</v>
+      </c>
+      <c r="E31" s="21" t="s">
+        <v>155</v>
+      </c>
+      <c r="F31" s="20" t="s">
+        <v>156</v>
+      </c>
+      <c r="G31" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="I31" s="21" t="s">
+        <v>153</v>
+      </c>
+      <c r="J31" s="20">
+        <v>33</v>
+      </c>
+      <c r="K31" s="26" t="s">
         <v>152</v>
-      </c>
-      <c r="F31" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="H31" s="25" t="s">
-        <v>79</v>
-      </c>
-      <c r="I31" s="19" t="s">
-        <v>150</v>
-      </c>
-      <c r="J31" s="18">
-        <v>33</v>
-      </c>
-      <c r="K31" s="22" t="s">
-        <v>352</v>
       </c>
       <c r="M31"/>
       <c r="N31"/>
@@ -2684,363 +3300,363 @@
       <c r="Q31"/>
       <c r="R31"/>
     </row>
-    <row r="32" spans="1:18" ht="36.75" thickBot="1">
+    <row r="32" ht="36.75" spans="1:11">
       <c r="A32" s="3"/>
       <c r="B32" s="8">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D32" s="12" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E32" s="13" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F32" s="12" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G32" s="13" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H32" s="12" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="I32" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J32" s="12">
         <v>1</v>
       </c>
       <c r="K32" s="12"/>
     </row>
-    <row r="33" spans="1:11" ht="36.75" thickBot="1">
+    <row r="33" ht="36.75" spans="1:11">
       <c r="A33" s="3"/>
       <c r="B33" s="8">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="C33" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="E33" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F33" s="10" t="s">
         <v>160</v>
       </c>
-      <c r="D33" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="E33" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>157</v>
-      </c>
       <c r="G33" s="11" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J33" s="10">
         <v>2</v>
       </c>
       <c r="K33" s="10"/>
     </row>
-    <row r="34" spans="1:11" ht="15.75" thickBot="1">
+    <row r="34" ht="15.75" spans="1:11">
       <c r="A34" s="3"/>
       <c r="B34" s="8">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F34" s="12" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="G34" s="13" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="I34" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J34" s="12">
         <v>1</v>
       </c>
       <c r="K34" s="12"/>
     </row>
-    <row r="35" spans="1:11" ht="15.75" thickBot="1">
+    <row r="35" ht="15.75" spans="1:11">
       <c r="A35" s="3"/>
       <c r="B35" s="8">
         <f t="shared" ref="B35:B66" si="1">ROW(B35)-ROW($B$2)</f>
         <v>33</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E35" s="11" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="G35" s="11" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J35" s="10">
         <v>1</v>
       </c>
       <c r="K35" s="10"/>
     </row>
-    <row r="36" spans="1:11" ht="15.75" thickBot="1">
+    <row r="36" ht="15.75" spans="1:11">
       <c r="A36" s="3"/>
       <c r="B36" s="8">
         <f t="shared" si="1"/>
         <v>34</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="D36" s="23" t="s">
-        <v>176</v>
-      </c>
-      <c r="E36" s="24" t="s">
-        <v>177</v>
-      </c>
-      <c r="F36" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="G36" s="24" t="s">
+      <c r="D36" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="H36" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="I36" s="23" t="s">
-        <v>149</v>
-      </c>
-      <c r="J36" s="23">
+      <c r="E36" s="16" t="s">
+        <v>180</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="G36" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="J36" s="15">
         <v>1</v>
       </c>
-      <c r="K36" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K36" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" spans="1:11">
       <c r="A37" s="3"/>
       <c r="B37" s="8">
         <f t="shared" si="1"/>
         <v>35</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D37" s="10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I37" s="11" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="J37" s="10">
         <v>1</v>
       </c>
       <c r="K37" s="10"/>
     </row>
-    <row r="38" spans="1:11" ht="24.75" thickBot="1">
+    <row r="38" ht="24.75" spans="1:11">
       <c r="A38" s="3"/>
       <c r="B38" s="8">
         <f t="shared" si="1"/>
         <v>36</v>
       </c>
       <c r="C38" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D38" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="F38" s="12" t="s">
         <v>186</v>
       </c>
-      <c r="E38" s="13" t="s">
-        <v>187</v>
-      </c>
-      <c r="F38" s="12" t="s">
-        <v>183</v>
-      </c>
       <c r="G38" s="13" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="H38" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I38" s="13" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="J38" s="12">
         <v>11</v>
       </c>
       <c r="K38" s="12"/>
     </row>
-    <row r="39" spans="1:11" ht="15.75" thickBot="1">
+    <row r="39" ht="15.75" spans="1:11">
       <c r="A39" s="3"/>
       <c r="B39" s="8">
         <f t="shared" si="1"/>
         <v>37</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D39" s="10" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I39" s="11" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="J39" s="10">
         <v>1</v>
       </c>
       <c r="K39" s="10"/>
     </row>
-    <row r="40" spans="1:11" ht="15.75" thickBot="1">
+    <row r="40" ht="15.75" spans="1:11">
       <c r="A40" s="3"/>
       <c r="B40" s="8">
         <f t="shared" si="1"/>
         <v>38</v>
       </c>
       <c r="C40" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D40" s="12" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F40" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G40" s="13" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I40" s="13" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="J40" s="12">
         <v>3</v>
       </c>
       <c r="K40" s="12"/>
     </row>
-    <row r="41" spans="1:11" ht="24.75" thickBot="1">
+    <row r="41" ht="24.75" spans="1:11">
       <c r="A41" s="3"/>
       <c r="B41" s="8">
         <f t="shared" si="1"/>
         <v>39</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D41" s="10" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G41" s="11" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H41" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I41" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="J41" s="10">
         <v>13</v>
       </c>
-      <c r="K41" s="20"/>
-    </row>
-    <row r="42" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K41" s="27"/>
+    </row>
+    <row r="42" ht="15.75" spans="1:11">
       <c r="A42" s="3"/>
       <c r="B42" s="8">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>203</v>
-      </c>
-      <c r="D42" s="23" t="s">
-        <v>204</v>
-      </c>
-      <c r="E42" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="F42" s="23" t="s">
-        <v>183</v>
-      </c>
-      <c r="G42" s="24" t="s">
         <v>206</v>
       </c>
-      <c r="H42" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="I42" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="J42" s="23">
+      <c r="D42" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="E42" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="G42" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J42" s="15">
         <v>1</v>
       </c>
-      <c r="K42" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K42" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" spans="1:11">
       <c r="A43" s="3"/>
       <c r="B43" s="8">
         <f t="shared" si="1"/>
@@ -3048,1152 +3664,1152 @@
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="10" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G43" s="11" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="H43" s="10" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="I43" s="11" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="J43" s="10">
         <v>6</v>
       </c>
       <c r="K43" s="10"/>
     </row>
-    <row r="44" spans="1:11" ht="15.75" thickBot="1">
+    <row r="44" ht="15.75" spans="1:11">
       <c r="A44" s="3"/>
       <c r="B44" s="8">
         <f t="shared" si="1"/>
         <v>42</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="D44" s="23" t="s">
-        <v>212</v>
-      </c>
-      <c r="E44" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="F44" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="G44" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="H44" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="I44" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="J44" s="23">
+      <c r="D44" s="15" t="s">
+        <v>215</v>
+      </c>
+      <c r="E44" s="16" t="s">
+        <v>203</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="G44" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="H44" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I44" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J44" s="15">
         <v>3</v>
       </c>
-      <c r="K44" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K44" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" spans="1:11">
       <c r="A45" s="3"/>
       <c r="B45" s="8">
         <f t="shared" si="1"/>
         <v>43</v>
       </c>
       <c r="C45" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D45" s="10" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G45" s="11" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H45" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I45" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="J45" s="10">
         <v>4</v>
       </c>
       <c r="K45" s="10"/>
     </row>
-    <row r="46" spans="1:11" ht="36.75" thickBot="1">
+    <row r="46" ht="36.75" spans="1:11">
       <c r="A46" s="3"/>
       <c r="B46" s="8">
         <f t="shared" si="1"/>
         <v>44</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D46" s="12" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="E46" s="13" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F46" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G46" s="13" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="H46" s="12" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="I46" s="13" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="J46" s="12">
         <v>2</v>
       </c>
       <c r="K46" s="12"/>
     </row>
-    <row r="47" spans="1:11" ht="15.75" thickBot="1">
+    <row r="47" ht="15.75" spans="1:11">
       <c r="A47" s="3"/>
       <c r="B47" s="8">
         <f t="shared" si="1"/>
         <v>45</v>
       </c>
       <c r="C47" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="D47" s="26" t="s">
-        <v>222</v>
-      </c>
-      <c r="E47" s="27" t="s">
-        <v>214</v>
-      </c>
-      <c r="F47" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="G47" s="27" t="s">
-        <v>215</v>
-      </c>
-      <c r="H47" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="I47" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="J47" s="26">
+      <c r="D47" s="23" t="s">
+        <v>225</v>
+      </c>
+      <c r="E47" s="24" t="s">
+        <v>217</v>
+      </c>
+      <c r="F47" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="G47" s="24" t="s">
+        <v>218</v>
+      </c>
+      <c r="H47" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="I47" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="J47" s="23">
         <v>2</v>
       </c>
-      <c r="K47" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K47" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="48" ht="15.75" spans="1:11">
       <c r="A48" s="3"/>
       <c r="B48" s="8">
         <f t="shared" si="1"/>
         <v>46</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="D48" s="23" t="s">
-        <v>223</v>
-      </c>
-      <c r="E48" s="24" t="s">
-        <v>224</v>
-      </c>
-      <c r="F48" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="G48" s="24" t="s">
-        <v>225</v>
-      </c>
-      <c r="H48" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="I48" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="J48" s="23">
+      <c r="D48" s="15" t="s">
+        <v>226</v>
+      </c>
+      <c r="E48" s="16" t="s">
+        <v>227</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="G48" s="16" t="s">
+        <v>228</v>
+      </c>
+      <c r="H48" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I48" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J48" s="15">
         <v>2</v>
       </c>
-      <c r="K48" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K48" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="49" ht="15.75" spans="1:11">
       <c r="A49" s="3"/>
       <c r="B49" s="8">
         <f t="shared" si="1"/>
         <v>47</v>
       </c>
       <c r="C49" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D49" s="10" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G49" s="11" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H49" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I49" s="11" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="J49" s="10">
         <v>1</v>
       </c>
       <c r="K49" s="10"/>
     </row>
-    <row r="50" spans="1:11" ht="15.75" thickBot="1">
+    <row r="50" ht="15.75" spans="1:11">
       <c r="A50" s="3"/>
       <c r="B50" s="8">
         <f t="shared" si="1"/>
         <v>48</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>180</v>
-      </c>
-      <c r="D50" s="23" t="s">
-        <v>230</v>
-      </c>
-      <c r="E50" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="F50" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="G50" s="24" t="s">
-        <v>209</v>
-      </c>
-      <c r="H50" s="23" t="s">
-        <v>210</v>
-      </c>
-      <c r="I50" s="24" t="s">
-        <v>149</v>
-      </c>
-      <c r="J50" s="23">
+      <c r="D50" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="E50" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="F50" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="G50" s="16" t="s">
+        <v>212</v>
+      </c>
+      <c r="H50" s="15" t="s">
+        <v>213</v>
+      </c>
+      <c r="I50" s="16" t="s">
+        <v>151</v>
+      </c>
+      <c r="J50" s="15">
         <v>1</v>
       </c>
-      <c r="K50" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" thickBot="1">
+      <c r="K50" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="51" ht="15.75" spans="1:11">
       <c r="A51" s="3"/>
       <c r="B51" s="8">
         <f t="shared" si="1"/>
         <v>49</v>
       </c>
       <c r="C51" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D51" s="10" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E51" s="11" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G51" s="11" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="H51" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I51" s="11" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="J51" s="10">
         <v>1</v>
       </c>
       <c r="K51" s="10"/>
     </row>
-    <row r="52" spans="1:11" ht="15.75" thickBot="1">
+    <row r="52" ht="15.75" spans="1:11">
       <c r="A52" s="3"/>
       <c r="B52" s="8">
         <f t="shared" si="1"/>
         <v>50</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D52" s="12" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="E52" s="13" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="F52" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H52" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I52" s="13" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="J52" s="12">
         <v>4</v>
       </c>
       <c r="K52" s="12"/>
     </row>
-    <row r="53" spans="1:11" ht="15.75" thickBot="1">
+    <row r="53" ht="15.75" spans="1:11">
       <c r="A53" s="3"/>
       <c r="B53" s="8">
         <f t="shared" si="1"/>
         <v>51</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D53" s="10" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="E53" s="11" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G53" s="11" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I53" s="11" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="J53" s="10">
         <v>1</v>
       </c>
       <c r="K53" s="10"/>
     </row>
-    <row r="54" spans="1:11" ht="15.75" thickBot="1">
+    <row r="54" ht="15.75" spans="1:11">
       <c r="A54" s="3"/>
       <c r="B54" s="8">
         <f t="shared" si="1"/>
         <v>52</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D54" s="12" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E54" s="13" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F54" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G54" s="13" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="H54" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I54" s="13" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="J54" s="12">
         <v>1</v>
       </c>
       <c r="K54" s="12"/>
     </row>
-    <row r="55" spans="1:11" ht="15.75" thickBot="1">
+    <row r="55" ht="15.75" spans="1:11">
       <c r="A55" s="3"/>
       <c r="B55" s="8">
         <f t="shared" si="1"/>
         <v>53</v>
       </c>
       <c r="C55" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="E55" s="11" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="H55" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="J55" s="10">
         <v>1</v>
       </c>
       <c r="K55" s="10"/>
     </row>
-    <row r="56" spans="1:11" ht="15.75" thickBot="1">
+    <row r="56" ht="15.75" spans="1:11">
       <c r="A56" s="3"/>
       <c r="B56" s="8">
         <f t="shared" si="1"/>
         <v>54</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="D56" s="12" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="E56" s="13" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="G56" s="13" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H56" s="12" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="I56" s="13" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="J56" s="12">
         <v>3</v>
       </c>
       <c r="K56" s="12"/>
     </row>
-    <row r="57" spans="1:11" ht="15.75" thickBot="1">
+    <row r="57" ht="15.75" spans="1:11">
       <c r="A57" s="3"/>
       <c r="B57" s="8">
         <f t="shared" si="1"/>
         <v>55</v>
       </c>
       <c r="C57" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="D57" s="26" t="s">
+        <v>206</v>
+      </c>
+      <c r="D57" s="23" t="s">
+        <v>258</v>
+      </c>
+      <c r="E57" s="24" t="s">
         <v>255</v>
       </c>
-      <c r="E57" s="27" t="s">
-        <v>252</v>
-      </c>
-      <c r="F57" s="26" t="s">
-        <v>183</v>
-      </c>
-      <c r="G57" s="27" t="s">
-        <v>253</v>
-      </c>
-      <c r="H57" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="I57" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="J57" s="26">
+      <c r="F57" s="23" t="s">
+        <v>186</v>
+      </c>
+      <c r="G57" s="24" t="s">
+        <v>256</v>
+      </c>
+      <c r="H57" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="I57" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="J57" s="23">
         <v>1</v>
       </c>
-      <c r="K57" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="24.75" thickBot="1">
+      <c r="K57" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="58" ht="24.75" spans="1:11">
       <c r="A58" s="3"/>
       <c r="B58" s="8">
         <f t="shared" si="1"/>
         <v>56</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D58" s="12" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="E58" s="13" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="G58" s="13" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="H58" s="12" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I58" s="13" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="J58" s="12">
         <v>1</v>
       </c>
       <c r="K58" s="12"/>
     </row>
-    <row r="59" spans="1:11" ht="24.75" thickBot="1">
+    <row r="59" ht="24.75" spans="1:11">
       <c r="A59" s="3"/>
       <c r="B59" s="8">
         <f t="shared" si="1"/>
         <v>57</v>
       </c>
       <c r="C59" s="9" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E59" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="F59" s="10" t="s">
+        <v>266</v>
+      </c>
+      <c r="G59" s="11" t="s">
+        <v>267</v>
+      </c>
+      <c r="H59" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="F59" s="10" t="s">
-        <v>263</v>
-      </c>
-      <c r="G59" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>259</v>
-      </c>
       <c r="I59" s="11" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="J59" s="10">
         <v>1</v>
       </c>
       <c r="K59" s="10"/>
     </row>
-    <row r="60" spans="1:11" ht="36.75" thickBot="1">
+    <row r="60" ht="36.75" spans="1:11">
       <c r="A60" s="3"/>
       <c r="B60" s="8">
         <f t="shared" si="1"/>
         <v>58</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="D60" s="12" t="s">
+        <v>269</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>270</v>
+      </c>
+      <c r="F60" s="12" t="s">
         <v>266</v>
       </c>
-      <c r="E60" s="13" t="s">
-        <v>267</v>
-      </c>
-      <c r="F60" s="12" t="s">
-        <v>263</v>
-      </c>
       <c r="G60" s="13" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="H60" s="12" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="I60" s="13" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="J60" s="12">
         <v>1</v>
       </c>
       <c r="K60" s="12"/>
     </row>
-    <row r="61" spans="1:11" ht="15.75" thickBot="1">
+    <row r="61" ht="15.75" spans="1:11">
       <c r="A61" s="3"/>
       <c r="B61" s="8">
         <f t="shared" si="1"/>
         <v>59</v>
       </c>
       <c r="C61" s="9" t="s">
-        <v>270</v>
-      </c>
-      <c r="D61" s="26" t="s">
-        <v>271</v>
-      </c>
-      <c r="E61" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="F61" s="26" t="s">
         <v>273</v>
       </c>
-      <c r="G61" s="27" t="s">
-        <v>273</v>
-      </c>
-      <c r="H61" s="26" t="s">
+      <c r="D61" s="23" t="s">
         <v>274</v>
       </c>
-      <c r="I61" s="27" t="s">
-        <v>149</v>
-      </c>
-      <c r="J61" s="26">
+      <c r="E61" s="24" t="s">
+        <v>275</v>
+      </c>
+      <c r="F61" s="23" t="s">
+        <v>276</v>
+      </c>
+      <c r="G61" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="H61" s="23" t="s">
+        <v>277</v>
+      </c>
+      <c r="I61" s="24" t="s">
+        <v>151</v>
+      </c>
+      <c r="J61" s="23">
         <v>1</v>
       </c>
-      <c r="K61" s="22" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" ht="36.75" thickBot="1">
+      <c r="K61" s="26" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="62" ht="36.75" spans="1:11">
       <c r="A62" s="3"/>
       <c r="B62" s="8">
         <f t="shared" si="1"/>
         <v>60</v>
       </c>
       <c r="C62" s="9" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D62" s="12" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="E62" s="13" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="F62" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="G62" s="13" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="H62" s="12" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="I62" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J62" s="12">
         <v>2</v>
       </c>
       <c r="K62" s="12"/>
     </row>
-    <row r="63" spans="1:11" ht="15.75" thickBot="1">
+    <row r="63" ht="15.75" spans="1:11">
       <c r="A63" s="3"/>
       <c r="B63" s="8">
         <f t="shared" si="1"/>
         <v>61</v>
       </c>
       <c r="C63" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D63" s="10" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="E63" s="11" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="F63" s="10" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="H63" s="10" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J63" s="10">
         <v>1</v>
       </c>
       <c r="K63" s="10"/>
     </row>
-    <row r="64" spans="1:11" ht="15.75" thickBot="1">
+    <row r="64" ht="15.75" spans="1:11">
       <c r="A64" s="3"/>
       <c r="B64" s="8">
         <f t="shared" si="1"/>
         <v>62</v>
       </c>
       <c r="C64" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D64" s="12" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E64" s="13" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F64" s="12" t="s">
+        <v>290</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>291</v>
+      </c>
+      <c r="H64" s="12" t="s">
         <v>287</v>
       </c>
-      <c r="G64" s="13" t="s">
-        <v>288</v>
-      </c>
-      <c r="H64" s="12" t="s">
-        <v>284</v>
-      </c>
       <c r="I64" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J64" s="12">
         <v>1</v>
       </c>
       <c r="K64" s="12"/>
     </row>
-    <row r="65" spans="1:11" ht="24.75" thickBot="1">
+    <row r="65" ht="24.75" spans="1:11">
       <c r="A65" s="3"/>
       <c r="B65" s="8">
         <f t="shared" si="1"/>
         <v>63</v>
       </c>
       <c r="C65" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D65" s="10" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E65" s="11" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F65" s="10" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="H65" s="10" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J65" s="10">
         <v>1</v>
       </c>
       <c r="K65" s="10"/>
     </row>
-    <row r="66" spans="1:11" ht="15.75" thickBot="1">
+    <row r="66" ht="15.75" spans="1:11">
       <c r="A66" s="3"/>
       <c r="B66" s="8">
         <f t="shared" si="1"/>
         <v>64</v>
       </c>
       <c r="C66" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D66" s="12" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E66" s="13" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F66" s="12" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="G66" s="13" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="H66" s="12" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="I66" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J66" s="12">
         <v>1</v>
       </c>
       <c r="K66" s="12"/>
     </row>
-    <row r="67" spans="1:11" ht="36.75" thickBot="1">
+    <row r="67" ht="36.75" spans="1:11">
       <c r="A67" s="3"/>
       <c r="B67" s="8">
         <f t="shared" ref="B67:B78" si="2">ROW(B67)-ROW($B$2)</f>
         <v>65</v>
       </c>
       <c r="C67" s="9" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D67" s="10" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="E67" s="11" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F67" s="10" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G67" s="11" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="H67" s="10" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="I67" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J67" s="10">
         <v>4</v>
       </c>
       <c r="K67" s="10"/>
     </row>
-    <row r="68" spans="1:11" ht="24.75" thickBot="1">
+    <row r="68" ht="24.75" spans="1:11">
       <c r="A68" s="3"/>
       <c r="B68" s="8">
         <f t="shared" si="2"/>
         <v>66</v>
       </c>
       <c r="C68" s="14" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E68" s="13" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G68" s="13" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="H68" s="12"/>
       <c r="I68" s="13" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J68" s="12">
         <v>1</v>
       </c>
       <c r="K68" s="12"/>
     </row>
-    <row r="69" spans="1:11" ht="15.75" thickBot="1">
+    <row r="69" ht="15.75" spans="1:11">
       <c r="A69" s="3"/>
       <c r="B69" s="8">
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
       <c r="C69" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D69" s="10" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="E69" s="11" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="F69" s="10" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="G69" s="11" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="H69" s="10" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I69" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J69" s="10">
         <v>1</v>
       </c>
       <c r="K69" s="10"/>
     </row>
-    <row r="70" spans="1:11" ht="15.75" thickBot="1">
+    <row r="70" ht="15.75" spans="1:11">
       <c r="A70" s="3"/>
       <c r="B70" s="8">
         <f t="shared" si="2"/>
         <v>68</v>
       </c>
       <c r="C70" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D70" s="12" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="E70" s="13" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="F70" s="12" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="G70" s="13" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I70" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J70" s="12">
         <v>1</v>
       </c>
       <c r="K70" s="12"/>
     </row>
-    <row r="71" spans="1:11" ht="15.75" thickBot="1">
+    <row r="71" ht="15.75" spans="1:11">
       <c r="A71" s="3"/>
       <c r="B71" s="8">
         <f t="shared" si="2"/>
         <v>69</v>
       </c>
       <c r="C71" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D71" s="10" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="E71" s="11" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F71" s="10" t="s">
+        <v>290</v>
+      </c>
+      <c r="G71" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="H71" s="10" t="s">
         <v>287</v>
       </c>
-      <c r="G71" s="11" t="s">
-        <v>318</v>
-      </c>
-      <c r="H71" s="10" t="s">
-        <v>284</v>
-      </c>
       <c r="I71" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J71" s="10">
         <v>1</v>
       </c>
       <c r="K71" s="10"/>
     </row>
-    <row r="72" spans="1:11" ht="15.75" thickBot="1">
+    <row r="72" ht="15.75" spans="1:11">
       <c r="A72" s="3"/>
       <c r="B72" s="8">
         <f t="shared" si="2"/>
         <v>70</v>
       </c>
       <c r="C72" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="E72" s="13" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F72" s="12" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="G72" s="13" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I72" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J72" s="12">
         <v>1</v>
       </c>
       <c r="K72" s="12"/>
     </row>
-    <row r="73" spans="1:11" ht="24.75" thickBot="1">
+    <row r="73" ht="24.75" spans="1:11">
       <c r="A73" s="3"/>
       <c r="B73" s="8">
         <f t="shared" si="2"/>
         <v>71</v>
       </c>
       <c r="C73" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D73" s="10" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="E73" s="11" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F73" s="10" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="G73" s="11" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="H73" s="10" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I73" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J73" s="10">
         <v>1</v>
       </c>
       <c r="K73" s="10"/>
     </row>
-    <row r="74" spans="1:11" ht="15.75" thickBot="1">
+    <row r="74" ht="15.75" spans="1:11">
       <c r="A74" s="3"/>
       <c r="B74" s="8">
         <f t="shared" si="2"/>
         <v>72</v>
       </c>
       <c r="C74" s="14" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D74" s="12" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E74" s="13" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F74" s="12" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="G74" s="13" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H74" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="I74" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J74" s="12">
         <v>1</v>
       </c>
       <c r="K74" s="12"/>
     </row>
-    <row r="75" spans="1:11" ht="15.75" thickBot="1">
+    <row r="75" ht="15.75" spans="1:11">
       <c r="A75" s="3"/>
       <c r="B75" s="8">
         <f t="shared" si="2"/>
         <v>73</v>
       </c>
       <c r="C75" s="9" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="D75" s="10" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E75" s="11" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F75" s="10" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="G75" s="11" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="H75" s="10" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="I75" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J75" s="10">
         <v>1</v>
       </c>
       <c r="K75" s="10"/>
     </row>
-    <row r="76" spans="1:11" ht="36.75" thickBot="1">
+    <row r="76" ht="36.75" spans="1:11">
       <c r="A76" s="3"/>
       <c r="B76" s="8">
         <f t="shared" si="2"/>
         <v>74</v>
       </c>
       <c r="C76" s="14" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="E76" s="13" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F76" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G76" s="13" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="H76" s="12" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="I76" s="13" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="J76" s="12">
         <v>1</v>
       </c>
       <c r="K76" s="12"/>
     </row>
-    <row r="77" spans="1:11" ht="24.75" thickBot="1">
+    <row r="77" ht="24.75" spans="1:11">
       <c r="A77" s="3"/>
       <c r="B77" s="8">
         <f t="shared" si="2"/>
         <v>75</v>
       </c>
       <c r="C77" s="9" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D77" s="10" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E77" s="11" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F77" s="10" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G77" s="11" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H77" s="10" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="I77" s="11" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J77" s="10">
         <v>1</v>
       </c>
       <c r="K77" s="10"/>
     </row>
-    <row r="78" spans="1:11" ht="15.75" thickBot="1">
+    <row r="78" ht="15.75" spans="1:11">
       <c r="A78" s="3"/>
       <c r="B78" s="8">
         <f t="shared" si="2"/>
         <v>76</v>
       </c>
       <c r="C78" s="9" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D78" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="E78" s="11" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="F78" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G78" s="11" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H78" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I78" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J78" s="10">
         <v>1</v>
@@ -4205,6 +4821,7 @@
     <mergeCell ref="I1:K1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>